<commit_message>
Fix craft realism: real material chains for cloth, alchemy, lumber, cooking.
Implements issue #92 P0+P1 (and broadens Dustgrain+dust cooking fillers):
- Cloth: pale-flax → linen-thread → linen-cloth; shade cotton thread for shade gear
- Alchemy/glass: distilled-pale for PH potions; river-sand → glass-bead; distilled-ash Ashlands+
- bloodbeam-lumber uses bark-strip (not Soft Pelt)
- Named cooking restores proteins/spices; breads stay grain-centric
- Gather/drop hooks for new bases; craft.ts supports OR material alternatives
</commit_message>
<xml_diff>
--- a/docs/legend-of-kek-item-manifest.xlsx
+++ b/docs/legend-of-kek-item-manifest.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K545"/>
+  <dimension ref="A1:K549"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -7142,10 +7142,14 @@
       </c>
       <c r="I149" s="4" t="inlineStr">
         <is>
-          <t>Craft: Woodworking Lv40 — requires Bloodbeam Log×2, Soft Pelt×1, Slag Dust×1</t>
-        </is>
-      </c>
-      <c r="J149" s="3" t="inlineStr"/>
+          <t>Craft: Woodworking Lv40 — requires Bloodbeam Log×2, Bark Strip×1, Slag Dust×1</t>
+        </is>
+      </c>
+      <c r="J149" s="3" t="inlineStr">
+        <is>
+          <t>P1: bark-strip not Soft Pelt</t>
+        </is>
+      </c>
       <c r="K149" s="3" t="inlineStr"/>
     </row>
     <row r="150">
@@ -12049,7 +12053,7 @@
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Needed</t>
         </is>
       </c>
       <c r="B252" s="3" t="inlineStr">
@@ -12087,10 +12091,14 @@
       </c>
       <c r="I252" s="4" t="inlineStr">
         <is>
-          <t>Craft: Clothcraft Lv1 — requires Shade Cotton×2 or Linen Scrap×3, Pale Dust×1</t>
-        </is>
-      </c>
-      <c r="J252" s="3" t="inlineStr"/>
+          <t>Craft: Clothcraft Lv1 — requires Linen Thread×3 or Linen Scrap×4, Pale Dust×1</t>
+        </is>
+      </c>
+      <c r="J252" s="3" t="inlineStr">
+        <is>
+          <t>P0: from linen-thread (or scrap recycle); shade-cotton removed</t>
+        </is>
+      </c>
       <c r="K252" s="3" t="inlineStr"/>
     </row>
     <row r="253">
@@ -12576,7 +12584,7 @@
       </c>
       <c r="C263" s="3" t="inlineStr">
         <is>
-          <t>Linen Thread×8</t>
+          <t>Linen Thread</t>
         </is>
       </c>
       <c r="D263" s="3" t="inlineStr">
@@ -12590,11 +12598,11 @@
         </is>
       </c>
       <c r="F263" s="3" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="G263" s="3" t="inlineStr">
         <is>
-          <t>filler</t>
+          <t>intermediate</t>
         </is>
       </c>
       <c r="H263" s="3" t="inlineStr">
@@ -12604,10 +12612,14 @@
       </c>
       <c r="I263" s="4" t="inlineStr">
         <is>
-          <t>Craft: Clothcraft Lv20 — requires Linen Cloth×1, Pale Dust×1</t>
-        </is>
-      </c>
-      <c r="J263" s="3" t="inlineStr"/>
+          <t>Craft: Clothcraft Lv1 — requires Pale Flax×2, Dead Fiber×1, Pale Dust×1</t>
+        </is>
+      </c>
+      <c r="J263" s="3" t="inlineStr">
+        <is>
+          <t>P0: fiber→thread (was reverse from cloth)</t>
+        </is>
+      </c>
       <c r="K263" s="3" t="inlineStr"/>
     </row>
     <row r="264">
@@ -12796,7 +12808,7 @@
       </c>
       <c r="I267" s="4" t="inlineStr">
         <is>
-          <t>Craft: Clothcraft Lv28 — requires Linen Cloth×1, Dead Fiber×1, Ash Dust×1</t>
+          <t>Craft: Clothcraft Lv28 — requires Linen Cloth×1, Shade Cotton×1, Ash Dust×1</t>
         </is>
       </c>
       <c r="J267" s="3" t="inlineStr"/>
@@ -12843,7 +12855,7 @@
       </c>
       <c r="I268" s="4" t="inlineStr">
         <is>
-          <t>Craft: Clothcraft Lv30 — requires Linen Cloth×3, Dead Fiber×1, Ash Dust×1</t>
+          <t>Craft: Clothcraft Lv30 — requires Linen Cloth×3, Shade Cotton Thread×1, Ash Dust×1</t>
         </is>
       </c>
       <c r="J268" s="3" t="inlineStr"/>
@@ -12890,7 +12902,7 @@
       </c>
       <c r="I269" s="4" t="inlineStr">
         <is>
-          <t>Craft: Clothcraft Lv32 — requires Linen Cloth×1, Dead Fiber×1, Ash Dust×1</t>
+          <t>Craft: Clothcraft Lv32 — requires Linen Cloth×1, Shade Cotton×1, Ash Dust×1</t>
         </is>
       </c>
       <c r="J269" s="3" t="inlineStr"/>
@@ -12937,7 +12949,7 @@
       </c>
       <c r="I270" s="4" t="inlineStr">
         <is>
-          <t>Craft: Clothcraft Lv34 — requires Linen Cloth×2, Dead Fiber×1, Ash Dust×1</t>
+          <t>Craft: Clothcraft Lv34 — requires Linen Cloth×2, Shade Cotton×1, Ash Dust×1</t>
         </is>
       </c>
       <c r="J270" s="3" t="inlineStr"/>
@@ -12984,7 +12996,7 @@
       </c>
       <c r="I271" s="4" t="inlineStr">
         <is>
-          <t>Craft: Clothcraft Lv36 — requires Linen Cloth×1, Dead Fiber×1, Ash Dust×1</t>
+          <t>Craft: Clothcraft Lv36 — requires Linen Cloth×1, Shade Cotton×1, Ash Dust×1</t>
         </is>
       </c>
       <c r="J271" s="3" t="inlineStr"/>
@@ -13054,7 +13066,7 @@
       </c>
       <c r="C273" s="3" t="inlineStr">
         <is>
-          <t>Ash Linen Thread×8</t>
+          <t>Shade Cotton Thread</t>
         </is>
       </c>
       <c r="D273" s="3" t="inlineStr">
@@ -13068,11 +13080,11 @@
         </is>
       </c>
       <c r="F273" s="3" t="n">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="G273" s="3" t="inlineStr">
         <is>
-          <t>filler</t>
+          <t>intermediate</t>
         </is>
       </c>
       <c r="H273" s="3" t="inlineStr">
@@ -13082,12 +13094,12 @@
       </c>
       <c r="I273" s="4" t="inlineStr">
         <is>
-          <t>Craft: Clothcraft Lv40 — requires Linen Cloth×1, Ash Dust×1</t>
+          <t>Craft: Clothcraft Lv25 — requires Shade Cotton×2, Ash Dust×1</t>
         </is>
       </c>
       <c r="J273" s="6" t="inlineStr">
         <is>
-          <t>renamed from v1 dup 'Linen Thread×8'</t>
+          <t>P0: renamed; cotton thread for shade gear</t>
         </is>
       </c>
       <c r="K273" s="3" t="inlineStr"/>
@@ -13231,10 +13243,14 @@
       </c>
       <c r="I276" s="4" t="inlineStr">
         <is>
-          <t>Craft: Clothcraft Lv45 — requires Silk Thread×3, Slag Dust×1</t>
-        </is>
-      </c>
-      <c r="J276" s="3" t="inlineStr"/>
+          <t>Craft: Clothcraft Lv45 — requires Spun Silk×1, Slag Dust×1</t>
+        </is>
+      </c>
+      <c r="J276" s="3" t="inlineStr">
+        <is>
+          <t>P1: consumes Spun Silk intermediate</t>
+        </is>
+      </c>
       <c r="K276" s="3" t="inlineStr"/>
     </row>
     <row r="277">
@@ -13579,7 +13595,7 @@
       </c>
       <c r="C284" s="3" t="inlineStr">
         <is>
-          <t>Silk Thread×8</t>
+          <t>Spun Silk</t>
         </is>
       </c>
       <c r="D284" s="3" t="inlineStr">
@@ -13593,11 +13609,11 @@
         </is>
       </c>
       <c r="F284" s="3" t="n">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="G284" s="3" t="inlineStr">
         <is>
-          <t>filler</t>
+          <t>intermediate</t>
         </is>
       </c>
       <c r="H284" s="3" t="inlineStr">
@@ -13607,10 +13623,14 @@
       </c>
       <c r="I284" s="4" t="inlineStr">
         <is>
-          <t>Craft: Clothcraft Lv60 — requires Silk Cloth×1, Slag Dust×1</t>
-        </is>
-      </c>
-      <c r="J284" s="3" t="inlineStr"/>
+          <t>Craft: Clothcraft Lv45 — requires Silk Thread×3, Slag Dust×1</t>
+        </is>
+      </c>
+      <c r="J284" s="3" t="inlineStr">
+        <is>
+          <t>P1: spun from base silk-thread (not from cloth)</t>
+        </is>
+      </c>
       <c r="K284" s="3" t="inlineStr"/>
     </row>
     <row r="285">
@@ -13752,10 +13772,14 @@
       </c>
       <c r="I287" s="4" t="inlineStr">
         <is>
-          <t>Craft: Clothcraft Lv65 — requires Velvet Dust×2, Silk Cloth×1, Bell Dust×1</t>
-        </is>
-      </c>
-      <c r="J287" s="3" t="inlineStr"/>
+          <t>Craft: Clothcraft Lv65 — requires Velvet Thread×3, Silk Cloth×1, Bell Dust×1</t>
+        </is>
+      </c>
+      <c r="J287" s="3" t="inlineStr">
+        <is>
+          <t>P1: from velvet-thread</t>
+        </is>
+      </c>
       <c r="K287" s="3" t="inlineStr"/>
     </row>
     <row r="288">
@@ -14104,7 +14128,7 @@
       </c>
       <c r="C295" s="3" t="inlineStr">
         <is>
-          <t>Velvet Thread×8</t>
+          <t>Velvet Thread</t>
         </is>
       </c>
       <c r="D295" s="3" t="inlineStr">
@@ -14118,11 +14142,11 @@
         </is>
       </c>
       <c r="F295" s="3" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="G295" s="3" t="inlineStr">
         <is>
-          <t>filler</t>
+          <t>intermediate</t>
         </is>
       </c>
       <c r="H295" s="3" t="inlineStr">
@@ -14132,10 +14156,14 @@
       </c>
       <c r="I295" s="4" t="inlineStr">
         <is>
-          <t>Craft: Clothcraft Lv80 — requires Velvet Cloth×1, Bell Dust×1</t>
-        </is>
-      </c>
-      <c r="J295" s="3" t="inlineStr"/>
+          <t>Craft: Clothcraft Lv60 — requires Velvet Fiber×2, Bell Dust×1</t>
+        </is>
+      </c>
+      <c r="J295" s="3" t="inlineStr">
+        <is>
+          <t>P1: fiber→thread</t>
+        </is>
+      </c>
       <c r="K295" s="3" t="inlineStr"/>
     </row>
     <row r="296">
@@ -17551,7 +17579,7 @@
     <row r="366">
       <c r="A366" s="5" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Needed</t>
         </is>
       </c>
       <c r="B366" s="3" t="inlineStr">
@@ -17589,10 +17617,14 @@
       </c>
       <c r="I366" s="4" t="inlineStr">
         <is>
-          <t>Craft: Goldsmithing Lv1 — requires Distilled Ash×1, Pale Dust×1</t>
-        </is>
-      </c>
-      <c r="J366" s="3" t="inlineStr"/>
+          <t>Craft: Goldsmithing Lv1 — requires River Sand×2, Potter's Clay×1, Pale Dust×1</t>
+        </is>
+      </c>
+      <c r="J366" s="3" t="inlineStr">
+        <is>
+          <t>P0: sand+clay kiln, not ash dust</t>
+        </is>
+      </c>
       <c r="K366" s="3" t="inlineStr"/>
     </row>
     <row r="367">
@@ -20335,7 +20367,7 @@
     <row r="422">
       <c r="A422" s="5" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Needed</t>
         </is>
       </c>
       <c r="B422" s="3" t="inlineStr">
@@ -20359,7 +20391,7 @@
         </is>
       </c>
       <c r="F422" s="3" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="G422" s="3" t="inlineStr">
         <is>
@@ -20373,10 +20405,14 @@
       </c>
       <c r="I422" s="4" t="inlineStr">
         <is>
-          <t>Craft: Alchemy Lv1 — requires Ash Dust×2</t>
-        </is>
-      </c>
-      <c r="J422" s="3" t="inlineStr"/>
+          <t>Craft: Alchemy Lv20 — requires Ash Dust×2, Antidote Root×1</t>
+        </is>
+      </c>
+      <c r="J422" s="3" t="inlineStr">
+        <is>
+          <t>P0: Ashlands+ intermediate (was PH L1 gate)</t>
+        </is>
+      </c>
       <c r="K422" s="3" t="inlineStr"/>
     </row>
     <row r="423">
@@ -20467,7 +20503,7 @@
       </c>
       <c r="I424" s="4" t="inlineStr">
         <is>
-          <t>Craft: Alchemy Lv5 — requires Distilled Ash×1, Dustgrain×1, Pale Dust×1</t>
+          <t>Craft: Alchemy Lv5 — requires Distilled Pale×1, Dustgrain×1, Pale Dust×1</t>
         </is>
       </c>
       <c r="J424" s="3" t="inlineStr"/>
@@ -20514,7 +20550,7 @@
       </c>
       <c r="I425" s="4" t="inlineStr">
         <is>
-          <t>Craft: Alchemy Lv7 — requires Distilled Ash×1, Pale Dust×1</t>
+          <t>Craft: Alchemy Lv7 — requires Distilled Pale×1, Pale Dust×1</t>
         </is>
       </c>
       <c r="J425" s="3" t="inlineStr"/>
@@ -20561,7 +20597,7 @@
       </c>
       <c r="I426" s="4" t="inlineStr">
         <is>
-          <t>Craft: Alchemy Lv9 — requires Distilled Ash×1, Pale Dust×1</t>
+          <t>Craft: Alchemy Lv9 — requires Distilled Pale×1, Pale Dust×1</t>
         </is>
       </c>
       <c r="J426" s="3" t="inlineStr"/>
@@ -20608,7 +20644,7 @@
       </c>
       <c r="I427" s="4" t="inlineStr">
         <is>
-          <t>Craft: Alchemy Lv11 — requires Distilled Ash×1, Pale Dust×1</t>
+          <t>Craft: Alchemy Lv11 — requires Distilled Pale×1, Pale Dust×1</t>
         </is>
       </c>
       <c r="J427" s="3" t="inlineStr"/>
@@ -20702,7 +20738,7 @@
       </c>
       <c r="I429" s="4" t="inlineStr">
         <is>
-          <t>Craft: Alchemy Lv14 — requires Distilled Ash×1, Pale Dust×1</t>
+          <t>Craft: Alchemy Lv14 — requires Distilled Pale×1, Pale Dust×1</t>
         </is>
       </c>
       <c r="J429" s="3" t="inlineStr"/>
@@ -20749,7 +20785,7 @@
       </c>
       <c r="I430" s="4" t="inlineStr">
         <is>
-          <t>Craft: Alchemy Lv16 — requires Distilled Ash×1, Pale Dust×1</t>
+          <t>Craft: Alchemy Lv16 — requires Distilled Pale×1, Pale Dust×1</t>
         </is>
       </c>
       <c r="J430" s="3" t="inlineStr"/>
@@ -23090,7 +23126,7 @@
     <row r="479">
       <c r="A479" s="5" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Needed</t>
         </is>
       </c>
       <c r="B479" s="3" t="inlineStr">
@@ -23128,7 +23164,7 @@
       </c>
       <c r="I479" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv3 — requires Dustgrain×1, Pale Dust×1</t>
+          <t>Craft: Cooking Lv3 — requires Rock Salt×1, Dustgrain×1, Pale Dust×1</t>
         </is>
       </c>
       <c r="J479" s="3" t="inlineStr"/>
@@ -23184,7 +23220,7 @@
     <row r="481">
       <c r="A481" s="5" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Needed</t>
         </is>
       </c>
       <c r="B481" s="3" t="inlineStr">
@@ -23222,7 +23258,7 @@
       </c>
       <c r="I481" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv7 — requires Dustgrain×1, Pale Dust×1</t>
+          <t>Craft: Cooking Lv7 — requires Fossil Minnow×2, Dustgrain×1, Pale Dust×1</t>
         </is>
       </c>
       <c r="J481" s="3" t="inlineStr"/>
@@ -23316,7 +23352,7 @@
       </c>
       <c r="I483" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv10 — requires Dustgrain×1, Pale Dust×1</t>
+          <t>Craft: Cooking Lv10 — requires Clay Crab×1, Dustgrain×2, Pale Dust×1</t>
         </is>
       </c>
       <c r="J483" s="3" t="inlineStr"/>
@@ -23363,7 +23399,7 @@
       </c>
       <c r="I484" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv12 — requires Dustgrain×1, Pale Dust×1</t>
+          <t>Craft: Cooking Lv12 — requires Dustgrain×2, Rock Salt×1, Pale Dust×1</t>
         </is>
       </c>
       <c r="J484" s="3" t="inlineStr"/>
@@ -23410,7 +23446,7 @@
       </c>
       <c r="I485" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv14 — requires Dustgrain×1, Pale Dust×1</t>
+          <t>Craft: Cooking Lv14 — requires Dustgrain×2, Pale Dust×1</t>
         </is>
       </c>
       <c r="J485" s="3" t="inlineStr"/>
@@ -23457,10 +23493,14 @@
       </c>
       <c r="I486" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv16 — requires Dustgrain×1, Pale Dust×1</t>
-        </is>
-      </c>
-      <c r="J486" s="3" t="inlineStr"/>
+          <t>Craft: Cooking Lv16 — requires Echo Carp×1, Rock Salt×1, Pale Dust×1</t>
+        </is>
+      </c>
+      <c r="J486" s="3" t="inlineStr">
+        <is>
+          <t>P1: protein restored (echo-carp soft-gates by zone)</t>
+        </is>
+      </c>
       <c r="K486" s="3" t="inlineStr"/>
     </row>
     <row r="487">
@@ -23504,7 +23544,7 @@
       </c>
       <c r="I487" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv18 — requires Dustgrain×1, Pale Dust×1</t>
+          <t>Craft: Cooking Lv18 — requires Fossil Minnow×1, Clay Crab×1, Dustgrain×1, Pale Dust×1</t>
         </is>
       </c>
       <c r="J487" s="3" t="inlineStr"/>
@@ -23598,7 +23638,7 @@
       </c>
       <c r="I489" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv22 — requires Dustgrain×1, Ash Dust×1</t>
+          <t>Craft: Cooking Lv22 — requires Antidote Root×1, Dustgrain×1, Ash Dust×1</t>
         </is>
       </c>
       <c r="J489" s="3" t="inlineStr"/>
@@ -23645,7 +23685,7 @@
       </c>
       <c r="I490" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv24 — requires Dustgrain×1, Ash Dust×1</t>
+          <t>Craft: Cooking Lv24 — requires Bone Chip×1, Dustgrain×1, Ash Dust×1</t>
         </is>
       </c>
       <c r="J490" s="3" t="inlineStr"/>
@@ -23739,7 +23779,7 @@
       </c>
       <c r="I492" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv27 — requires Dustgrain×1, Ash Dust×1</t>
+          <t>Craft: Cooking Lv27 — requires Dustgrain×2, Rock Salt×1, Ash Dust×1</t>
         </is>
       </c>
       <c r="J492" s="3" t="inlineStr"/>
@@ -23786,7 +23826,7 @@
       </c>
       <c r="I493" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv29 — requires Dustgrain×1, Ash Dust×1</t>
+          <t>Craft: Cooking Lv29 — requires Bone Chip×2, Dustgrain×1, Ash Dust×1</t>
         </is>
       </c>
       <c r="J493" s="3" t="inlineStr"/>
@@ -23833,10 +23873,14 @@
       </c>
       <c r="I494" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv31 — requires Dustgrain×1, Ash Dust×1</t>
-        </is>
-      </c>
-      <c r="J494" s="3" t="inlineStr"/>
+          <t>Craft: Cooking Lv31 — requires Dried Ration Scrap×1, Dustgrain×1, Ash Dust×1</t>
+        </is>
+      </c>
+      <c r="J494" s="3" t="inlineStr">
+        <is>
+          <t>ration-style starter plate</t>
+        </is>
+      </c>
       <c r="K494" s="3" t="inlineStr"/>
     </row>
     <row r="495">
@@ -23880,7 +23924,7 @@
       </c>
       <c r="I495" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv33 — requires Dustgrain×1, Ash Dust×1</t>
+          <t>Craft: Cooking Lv33 — requires Bone Chip×1, Fossil Minnow×1, Ash Dust×1</t>
         </is>
       </c>
       <c r="J495" s="3" t="inlineStr"/>
@@ -23927,7 +23971,7 @@
       </c>
       <c r="I496" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv35 — requires Dustgrain×1, Ash Dust×1</t>
+          <t>Craft: Cooking Lv35 — requires Glass Bead×1, Dustgrain×1, Ash Dust×1</t>
         </is>
       </c>
       <c r="J496" s="3" t="inlineStr"/>
@@ -23974,7 +24018,7 @@
       </c>
       <c r="I497" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv37 — requires Dustgrain×1, Ash Dust×1</t>
+          <t>Craft: Cooking Lv37 — requires Clay Crab×1, Fossil Minnow×1, Dustgrain×1, Ash Dust×1</t>
         </is>
       </c>
       <c r="J497" s="3" t="inlineStr"/>
@@ -24021,7 +24065,7 @@
       </c>
       <c r="I498" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv39 — requires Dustgrain×1, Ash Dust×1</t>
+          <t>Craft: Cooking Lv39 — requires Fossil Minnow×2, Rock Salt×1, Ash Dust×1</t>
         </is>
       </c>
       <c r="J498" s="3" t="inlineStr"/>
@@ -24115,7 +24159,7 @@
       </c>
       <c r="I500" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv42 — requires Dustgrain×1, Slag Dust×1</t>
+          <t>Craft: Cooking Lv42 — requires Dustgrain×2, Rock Salt×1, Slag Dust×1</t>
         </is>
       </c>
       <c r="J500" s="3" t="inlineStr"/>
@@ -24162,7 +24206,7 @@
       </c>
       <c r="I501" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv44 — requires Dustgrain×1, Slag Dust×1</t>
+          <t>Craft: Cooking Lv44 — requires Fossil Minnow×1, Dustgrain×1, Slag Dust×1</t>
         </is>
       </c>
       <c r="J501" s="3" t="inlineStr"/>
@@ -24256,7 +24300,7 @@
       </c>
       <c r="I503" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv47 — requires Dustgrain×1, Slag Dust×1</t>
+          <t>Craft: Cooking Lv47 — requires Fossil Minnow×2, Dustgrain×1, Slag Dust×1</t>
         </is>
       </c>
       <c r="J503" s="6" t="inlineStr">
@@ -24354,7 +24398,7 @@
       </c>
       <c r="I505" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv50 — requires Dustgrain×1, Slag Dust×1</t>
+          <t>Craft: Cooking Lv50 — requires Clay Crab×1, Dustgrain×2, Slag Dust×1</t>
         </is>
       </c>
       <c r="J505" s="6" t="inlineStr">
@@ -24405,7 +24449,7 @@
       </c>
       <c r="I506" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv52 — requires Dustgrain×1, Slag Dust×1</t>
+          <t>Craft: Cooking Lv52 — requires Dustgrain×2, Rock Salt×1, Slag Dust×1</t>
         </is>
       </c>
       <c r="J506" s="6" t="inlineStr">
@@ -24456,7 +24500,7 @@
       </c>
       <c r="I507" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv54 — requires Dustgrain×1, Slag Dust×1</t>
+          <t>Craft: Cooking Lv54 — requires Dustgrain×2, Slag Dust×1</t>
         </is>
       </c>
       <c r="J507" s="6" t="inlineStr">
@@ -24507,7 +24551,7 @@
       </c>
       <c r="I508" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv56 — requires Dustgrain×1, Slag Dust×1</t>
+          <t>Craft: Cooking Lv56 — requires Echo Carp×1, Rock Salt×1, Slag Dust×1</t>
         </is>
       </c>
       <c r="J508" s="6" t="inlineStr">
@@ -24558,7 +24602,7 @@
       </c>
       <c r="I509" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv58 — requires Dustgrain×1, Slag Dust×1</t>
+          <t>Craft: Cooking Lv58 — requires Fossil Minnow×1, Clay Crab×1, Dustgrain×1, Slag Dust×1</t>
         </is>
       </c>
       <c r="J509" s="6" t="inlineStr">
@@ -24609,7 +24653,7 @@
       </c>
       <c r="I510" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv60 — requires Dustgrain×1, Slag Dust×1</t>
+          <t>Craft: Cooking Lv60 — requires Glass Eel×1, Bitter Spice×1, Slag Dust×1</t>
         </is>
       </c>
       <c r="J510" s="3" t="inlineStr"/>
@@ -24656,7 +24700,7 @@
       </c>
       <c r="I511" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv62 — requires Dustgrain×1, Bell Dust×1</t>
+          <t>Craft: Cooking Lv62 — requires Antidote Root×1, Echo Extract×1, Bell Dust×1</t>
         </is>
       </c>
       <c r="J511" s="6" t="inlineStr">
@@ -24707,7 +24751,7 @@
       </c>
       <c r="I512" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv64 — requires Dustgrain×1, Bell Dust×1</t>
+          <t>Craft: Cooking Lv64 — requires Bone Chip×1, Echo Carp×1, Bell Dust×1</t>
         </is>
       </c>
       <c r="J512" s="6" t="inlineStr">
@@ -24805,7 +24849,7 @@
       </c>
       <c r="I514" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv67 — requires Dustgrain×1, Bell Dust×1</t>
+          <t>Craft: Cooking Lv67 — requires Dustgrain×2, Rock Salt×1, Bell Dust×1</t>
         </is>
       </c>
       <c r="J514" s="6" t="inlineStr">
@@ -24856,7 +24900,7 @@
       </c>
       <c r="I515" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv69 — requires Dustgrain×1, Bell Dust×1</t>
+          <t>Craft: Cooking Lv69 — requires Bone Chip×2, Dustgrain×1, Bell Dust×1</t>
         </is>
       </c>
       <c r="J515" s="6" t="inlineStr">
@@ -24954,7 +24998,7 @@
       </c>
       <c r="I517" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv72 — requires Dustgrain×1, Bell Dust×1</t>
+          <t>Craft: Cooking Lv72 — requires Rock Salt×2, Bell Dust×1</t>
         </is>
       </c>
       <c r="J517" s="3" t="inlineStr"/>
@@ -25001,7 +25045,7 @@
       </c>
       <c r="I518" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv74 — requires Dustgrain×1, Bell Dust×1</t>
+          <t>Craft: Cooking Lv74 — requires Dustgrain×3, Rock Salt×1, Bell Dust×1</t>
         </is>
       </c>
       <c r="J518" s="6" t="inlineStr">
@@ -25052,7 +25096,7 @@
       </c>
       <c r="I519" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv76 — requires Dustgrain×1, Bell Dust×1</t>
+          <t>Craft: Cooking Lv76 — requires Desiccated Hide×1, Rock Salt×1, Bell Dust×1</t>
         </is>
       </c>
       <c r="J519" s="6" t="inlineStr">
@@ -25103,7 +25147,7 @@
       </c>
       <c r="I520" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv78 — requires Dustgrain×1, Bell Dust×1</t>
+          <t>Craft: Cooking Lv78 — requires Echo Carp×1, Clay Crab×1, Bell Dust×1</t>
         </is>
       </c>
       <c r="J520" s="3" t="inlineStr"/>
@@ -25150,7 +25194,7 @@
       </c>
       <c r="I521" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv80 — requires Dustgrain×1, Bell Dust×1</t>
+          <t>Craft: Cooking Lv80 — requires Rock Salt×2, Bell Dust×1</t>
         </is>
       </c>
       <c r="J521" s="3" t="inlineStr"/>
@@ -25197,7 +25241,7 @@
       </c>
       <c r="I522" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv82 — requires Dustgrain×1, Throne Dust×1</t>
+          <t>Craft: Cooking Lv82 — requires Dustgrain×2, Rock Salt×1, Throne Dust×1</t>
         </is>
       </c>
       <c r="J522" s="6" t="inlineStr">
@@ -25248,7 +25292,7 @@
       </c>
       <c r="I523" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv84 — requires Dustgrain×1, Throne Dust×1</t>
+          <t>Craft: Cooking Lv84 — requires Echo Carp×1, Dustgrain×1, Throne Dust×1</t>
         </is>
       </c>
       <c r="J523" s="6" t="inlineStr">
@@ -25299,7 +25343,7 @@
       </c>
       <c r="I524" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv86 — requires Dustgrain×1, Throne Dust×1</t>
+          <t>Craft: Cooking Lv86 — requires Scale Hide×1, Rock Salt×1, Throne Dust×1</t>
         </is>
       </c>
       <c r="J524" s="3" t="inlineStr"/>
@@ -25346,7 +25390,7 @@
       </c>
       <c r="I525" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv88 — requires Dustgrain×1, Throne Dust×1</t>
+          <t>Craft: Cooking Lv88 — requires Bone Chip×2, Dustgrain×1, Throne Dust×1</t>
         </is>
       </c>
       <c r="J525" s="3" t="inlineStr"/>
@@ -25440,7 +25484,7 @@
       </c>
       <c r="I527" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv92 — requires Dustgrain×1, Throne Dust×1</t>
+          <t>Craft: Cooking Lv92 — requires Dustgrain×2, Rock Salt×1, Throne Dust×1</t>
         </is>
       </c>
       <c r="J527" s="6" t="inlineStr">
@@ -25491,7 +25535,7 @@
       </c>
       <c r="I528" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv94 — requires Dustgrain×1, Throne Dust×1</t>
+          <t>Craft: Cooking Lv94 — requires Dustgrain×2, Throne Dust×1</t>
         </is>
       </c>
       <c r="J528" s="6" t="inlineStr">
@@ -25542,7 +25586,7 @@
       </c>
       <c r="I529" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv96 — requires Dustgrain×1, Throne Dust×1</t>
+          <t>Craft: Cooking Lv96 — requires Echo Carp×1, Rock Salt×1, Throne Dust×1</t>
         </is>
       </c>
       <c r="J529" s="6" t="inlineStr">
@@ -25593,7 +25637,7 @@
       </c>
       <c r="I530" s="4" t="inlineStr">
         <is>
-          <t>Craft: Cooking Lv98 — requires Dustgrain×1, Throne Dust×1</t>
+          <t>Craft: Cooking Lv98 — requires Echo Carp×1, Glass Eel×1, Dustgrain×1, Throne Dust×1</t>
         </is>
       </c>
       <c r="J530" s="6" t="inlineStr">
@@ -26307,6 +26351,217 @@
       </c>
       <c r="J545" s="3" t="inlineStr"/>
       <c r="K545" s="3" t="inlineStr"/>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>pale-flax</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>Pale Flax</t>
+        </is>
+      </c>
+      <c r="D546" t="inlineStr">
+        <is>
+          <t>Base Precursor</t>
+        </is>
+      </c>
+      <c r="E546" t="inlineStr">
+        <is>
+          <t>Fiber/cloth scrap</t>
+        </is>
+      </c>
+      <c r="G546" t="inlineStr">
+        <is>
+          <t>base</t>
+        </is>
+      </c>
+      <c r="H546" t="inlineStr">
+        <is>
+          <t>Mat</t>
+        </is>
+      </c>
+      <c r="I546" t="inlineStr">
+        <is>
+          <t>Harvest — Pale Hollow scrubland (flax stands / fiber thickets)</t>
+        </is>
+      </c>
+      <c r="J546" t="inlineStr">
+        <is>
+          <t>P0: linen precursor</t>
+        </is>
+      </c>
+      <c r="K546" t="inlineStr">
+        <is>
+          <t>craft-realism</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>river-sand</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>River Sand</t>
+        </is>
+      </c>
+      <c r="D547" t="inlineStr">
+        <is>
+          <t>Base Precursor</t>
+        </is>
+      </c>
+      <c r="E547" t="inlineStr">
+        <is>
+          <t>Stone/clay</t>
+        </is>
+      </c>
+      <c r="G547" t="inlineStr">
+        <is>
+          <t>base</t>
+        </is>
+      </c>
+      <c r="H547" t="inlineStr">
+        <is>
+          <t>Mat</t>
+        </is>
+      </c>
+      <c r="I547" t="inlineStr">
+        <is>
+          <t>Harvest — Pale Hollow riverbank clay banks</t>
+        </is>
+      </c>
+      <c r="J547" t="inlineStr">
+        <is>
+          <t>P0: glass precursor</t>
+        </is>
+      </c>
+      <c r="K547" t="inlineStr">
+        <is>
+          <t>craft-realism</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>velvet-fiber</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>Velvet Fiber</t>
+        </is>
+      </c>
+      <c r="D548" t="inlineStr">
+        <is>
+          <t>Base Precursor</t>
+        </is>
+      </c>
+      <c r="E548" t="inlineStr">
+        <is>
+          <t>Fiber/cloth scrap</t>
+        </is>
+      </c>
+      <c r="G548" t="inlineStr">
+        <is>
+          <t>base</t>
+        </is>
+      </c>
+      <c r="H548" t="inlineStr">
+        <is>
+          <t>Mat</t>
+        </is>
+      </c>
+      <c r="I548" t="inlineStr">
+        <is>
+          <t>Drop — Bellmarsh scale/velvet foes</t>
+        </is>
+      </c>
+      <c r="J548" t="inlineStr">
+        <is>
+          <t>P1: spinnable velvet</t>
+        </is>
+      </c>
+      <c r="K548" t="inlineStr">
+        <is>
+          <t>craft-realism</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>distilled-pale</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>Distilled Pale</t>
+        </is>
+      </c>
+      <c r="D549" t="inlineStr">
+        <is>
+          <t>Crafted</t>
+        </is>
+      </c>
+      <c r="E549" t="inlineStr">
+        <is>
+          <t>Alchemy</t>
+        </is>
+      </c>
+      <c r="F549" t="n">
+        <v>1</v>
+      </c>
+      <c r="G549" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="H549" t="inlineStr">
+        <is>
+          <t>Mat</t>
+        </is>
+      </c>
+      <c r="I549" t="inlineStr">
+        <is>
+          <t>Craft: Alchemy Lv1 — requires Pale Dust×2, Antidote Root×1</t>
+        </is>
+      </c>
+      <c r="J549" t="inlineStr">
+        <is>
+          <t>P0: PH alchemy intermediate</t>
+        </is>
+      </c>
+      <c r="K549" t="inlineStr">
+        <is>
+          <t>craft-realism</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K545"/>

</xml_diff>

<commit_message>
Add chainmail body armor: rare 1% Ruin Dweller drop.
ilvl 10 (+5 STR/DEX/AGI, +10 DEF) for knight/fighter/cleric/rogue/battlemage; icons in public+assets; rareDrops schema on Pale Hollow mobs.
</commit_message>
<xml_diff>
--- a/docs/legend-of-kek-item-manifest.xlsx
+++ b/docs/legend-of-kek-item-manifest.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K550"/>
+  <dimension ref="A1:K551"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -26682,6 +26682,61 @@
       <c r="J550" t="inlineStr">
         <is>
           <t>P2: Ashlands stone-scale (was Scale Leather L65 / Bellmarsh softlock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>chainmail</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>Chainmail</t>
+        </is>
+      </c>
+      <c r="D551" t="inlineStr">
+        <is>
+          <t>Drop</t>
+        </is>
+      </c>
+      <c r="E551" t="inlineStr">
+        <is>
+          <t>Smithing</t>
+        </is>
+      </c>
+      <c r="F551" t="n">
+        <v>10</v>
+      </c>
+      <c r="G551" t="inlineStr">
+        <is>
+          <t>equipment</t>
+        </is>
+      </c>
+      <c r="H551" t="inlineStr">
+        <is>
+          <t>Knight/Fighter/Cleric/Rogue/BM</t>
+        </is>
+      </c>
+      <c r="I551" t="inlineStr">
+        <is>
+          <t>Drop — Ruin Dweller (1%), Pale Hollow</t>
+        </is>
+      </c>
+      <c r="J551" t="inlineStr">
+        <is>
+          <t>Rare body armor ilvl10</t>
+        </is>
+      </c>
+      <c r="K551" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>

</xml_diff>